<commit_message>
APRESENTAÇÃO AMANHÃ PARA LEILA - COMISSÕES POR RECEBIMENTO NÃO FUNCIONAL - NENHUMA ALTERAÇÃO SOLICITADA FEITA AINDA - CRISE TOTAL
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_08_2025.xlsx
+++ b/Calculo_Comissoes_08_2025.xlsx
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO22"/>
+  <dimension ref="A1:BO17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -924,25 +924,25 @@
         <v>0.1</v>
       </c>
       <c r="N2" s="11" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="O2" s="12" t="n">
         <v>0.4</v>
       </c>
       <c r="P2" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q2" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R2" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S2" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T2" s="12" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="U2" s="13" t="n">
         <v>0.3</v>
@@ -1016,7 +1016,7 @@
         <v>0.25</v>
       </c>
       <c r="BN2" t="n">
-        <v>0.172</v>
+        <v>0.142</v>
       </c>
     </row>
     <row r="3">
@@ -1078,25 +1078,25 @@
         <v>0.2</v>
       </c>
       <c r="N3" s="11" t="n">
-        <v>0.608</v>
+        <v>0.518</v>
       </c>
       <c r="O3" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="P3" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q3" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R3" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S3" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T3" s="12" t="n">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
       <c r="U3" s="13" t="n">
         <v>0.4</v>
@@ -1170,7 +1170,7 @@
         <v>0.5</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.304</v>
+        <v>0.259</v>
       </c>
     </row>
     <row r="4">
@@ -1232,25 +1232,25 @@
         <v>0.2</v>
       </c>
       <c r="N4" s="11" t="n">
-        <v>0.6320000000000001</v>
+        <v>0.512</v>
       </c>
       <c r="O4" s="12" t="n">
         <v>0.4</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q4" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R4" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S4" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T4" s="12" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="U4" s="13" t="n">
         <v>0.4</v>
@@ -1324,7 +1324,7 @@
         <v>0.5</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.3160000000000001</v>
+        <v>0.256</v>
       </c>
     </row>
     <row r="5">
@@ -1386,7 +1386,7 @@
         <v>0.15</v>
       </c>
       <c r="N5" s="11" t="n">
-        <v>0.52</v>
+        <v>0.4</v>
       </c>
       <c r="O5" s="12" t="inlineStr"/>
       <c r="P5" s="12" t="inlineStr"/>
@@ -1404,19 +1404,19 @@
         <v>0.4</v>
       </c>
       <c r="AB5" s="14" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="AC5" s="14" t="n">
         <v>100</v>
       </c>
       <c r="AD5" s="14" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="AE5" s="14" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="AF5" s="14" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="AG5" s="15" t="n">
         <v>0.6</v>
@@ -1466,7 +1466,7 @@
         <v>0.375</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.195</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="6">
@@ -1528,7 +1528,7 @@
         <v>0.15</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="O6" s="12" t="inlineStr"/>
       <c r="P6" s="12" t="inlineStr"/>
@@ -1546,19 +1546,19 @@
         <v>0.6</v>
       </c>
       <c r="AB6" s="14" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="AC6" s="14" t="n">
         <v>100</v>
       </c>
       <c r="AD6" s="14" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="AE6" s="14" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="AF6" s="14" t="n">
-        <v>0.6</v>
+        <v>0.42</v>
       </c>
       <c r="AG6" s="15" t="n">
         <v>0.4</v>
@@ -1608,7 +1608,7 @@
         <v>0.375</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.255</v>
+        <v>0.1875</v>
       </c>
     </row>
     <row r="7">
@@ -1670,25 +1670,25 @@
         <v>0.1</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>0.46</v>
+        <v>0.34</v>
       </c>
       <c r="O7" s="12" t="n">
         <v>0.4</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q7" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R7" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S7" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T7" s="12" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="U7" s="13" t="n">
         <v>0.3</v>
@@ -1762,7 +1762,7 @@
         <v>0.1</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.04600000000000001</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="8">
@@ -1824,25 +1824,25 @@
         <v>0.2</v>
       </c>
       <c r="N8" s="11" t="n">
-        <v>0.38</v>
+        <v>0.29</v>
       </c>
       <c r="O8" s="12" t="n">
         <v>0.3</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q8" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R8" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S8" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T8" s="12" t="n">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
       <c r="U8" s="13" t="n">
         <v>0.4</v>
@@ -1916,7 +1916,7 @@
         <v>0.2</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.07600000000000001</v>
+        <v>0.05800000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -1978,25 +1978,25 @@
         <v>0.2</v>
       </c>
       <c r="N9" s="11" t="n">
-        <v>0.48</v>
+        <v>0.36</v>
       </c>
       <c r="O9" s="12" t="n">
         <v>0.4</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="Q9" s="12" t="n">
         <v>100</v>
       </c>
       <c r="R9" s="12" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="S9" s="12" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="T9" s="12" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="U9" s="13" t="n">
         <v>0.4</v>
@@ -2070,7 +2070,7 @@
         <v>0.2</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.09600000000000002</v>
+        <v>0.07199999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -2132,7 +2132,7 @@
         <v>0.15</v>
       </c>
       <c r="N10" s="11" t="n">
-        <v>0.52</v>
+        <v>0.4</v>
       </c>
       <c r="O10" s="12" t="inlineStr"/>
       <c r="P10" s="12" t="inlineStr"/>
@@ -2150,19 +2150,19 @@
         <v>0.4</v>
       </c>
       <c r="AB10" s="14" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="AC10" s="14" t="n">
         <v>100</v>
       </c>
       <c r="AD10" s="14" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="AE10" s="14" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="AF10" s="14" t="n">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="AG10" s="15" t="n">
         <v>0.6</v>
@@ -2212,7 +2212,7 @@
         <v>0.15</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.078</v>
+        <v>0.05999999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -2274,7 +2274,7 @@
         <v>0.15</v>
       </c>
       <c r="N11" s="11" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="O11" s="12" t="inlineStr"/>
       <c r="P11" s="12" t="inlineStr"/>
@@ -2292,19 +2292,19 @@
         <v>0.6</v>
       </c>
       <c r="AB11" s="14" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="AC11" s="14" t="n">
         <v>100</v>
       </c>
       <c r="AD11" s="14" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="AE11" s="14" t="n">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="AF11" s="14" t="n">
-        <v>0.6</v>
+        <v>0.42</v>
       </c>
       <c r="AG11" s="15" t="n">
         <v>0.4</v>
@@ -2354,7 +2354,7 @@
         <v>0.15</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.102</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="12">
@@ -3222,752 +3222,6 @@
         <v>0.525</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Paulo Negrão</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Diretor</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>100001</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>PROD100002</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Produto de Teste - Processo 100002</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>SSO</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Detector Portátil</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>MicroClip</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>50</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N18" s="11" t="n">
-        <v>0.6879999999999999</v>
-      </c>
-      <c r="O18" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P18" s="12" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q18" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R18" s="12" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T18" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="U18" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="V18" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="W18" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X18" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Y18" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Z18" s="13" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="AA18" s="14" t="inlineStr"/>
-      <c r="AB18" s="14" t="inlineStr"/>
-      <c r="AC18" s="14" t="inlineStr"/>
-      <c r="AD18" s="14" t="inlineStr"/>
-      <c r="AE18" s="14" t="inlineStr"/>
-      <c r="AF18" s="14" t="inlineStr"/>
-      <c r="AG18" s="15" t="inlineStr"/>
-      <c r="AH18" s="15" t="inlineStr"/>
-      <c r="AI18" s="15" t="inlineStr"/>
-      <c r="AJ18" s="15" t="inlineStr"/>
-      <c r="AK18" s="15" t="inlineStr"/>
-      <c r="AL18" s="15" t="inlineStr"/>
-      <c r="AM18" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN18" s="16" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AO18" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP18" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AQ18" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AR18" s="16" t="n">
-        <v>0.228</v>
-      </c>
-      <c r="AS18" s="17" t="inlineStr"/>
-      <c r="AT18" s="17" t="inlineStr"/>
-      <c r="AU18" s="17" t="inlineStr"/>
-      <c r="AV18" s="17" t="inlineStr"/>
-      <c r="AW18" s="17" t="inlineStr"/>
-      <c r="AX18" s="17" t="inlineStr"/>
-      <c r="AY18" s="18" t="inlineStr"/>
-      <c r="AZ18" s="18" t="inlineStr"/>
-      <c r="BA18" s="18" t="inlineStr"/>
-      <c r="BB18" s="18" t="inlineStr"/>
-      <c r="BC18" s="18" t="inlineStr"/>
-      <c r="BD18" s="18" t="inlineStr"/>
-      <c r="BE18" s="18" t="inlineStr"/>
-      <c r="BF18" s="19" t="inlineStr"/>
-      <c r="BG18" s="19" t="inlineStr"/>
-      <c r="BH18" s="19" t="inlineStr"/>
-      <c r="BI18" s="19" t="inlineStr"/>
-      <c r="BJ18" s="19" t="inlineStr"/>
-      <c r="BK18" s="19" t="inlineStr"/>
-      <c r="BL18" s="19" t="inlineStr"/>
-      <c r="BM18" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="BN18" t="n">
-        <v>0.172</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>C002</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Antônio Rosa</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Gerente Geral</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>100001</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PROD100002</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Produto de Teste - Processo 100002</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>SSO</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Detector Portátil</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>MicroClip</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>50</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N19" s="11" t="n">
-        <v>0.608</v>
-      </c>
-      <c r="O19" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P19" s="12" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q19" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R19" s="12" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T19" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="U19" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V19" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="W19" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X19" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Y19" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Z19" s="13" t="n">
-        <v>0.08000000000000002</v>
-      </c>
-      <c r="AA19" s="14" t="inlineStr"/>
-      <c r="AB19" s="14" t="inlineStr"/>
-      <c r="AC19" s="14" t="inlineStr"/>
-      <c r="AD19" s="14" t="inlineStr"/>
-      <c r="AE19" s="14" t="inlineStr"/>
-      <c r="AF19" s="14" t="inlineStr"/>
-      <c r="AG19" s="15" t="inlineStr"/>
-      <c r="AH19" s="15" t="inlineStr"/>
-      <c r="AI19" s="15" t="inlineStr"/>
-      <c r="AJ19" s="15" t="inlineStr"/>
-      <c r="AK19" s="15" t="inlineStr"/>
-      <c r="AL19" s="15" t="inlineStr"/>
-      <c r="AM19" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN19" s="16" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AO19" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP19" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AQ19" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AR19" s="16" t="n">
-        <v>0.228</v>
-      </c>
-      <c r="AS19" s="17" t="inlineStr"/>
-      <c r="AT19" s="17" t="inlineStr"/>
-      <c r="AU19" s="17" t="inlineStr"/>
-      <c r="AV19" s="17" t="inlineStr"/>
-      <c r="AW19" s="17" t="inlineStr"/>
-      <c r="AX19" s="17" t="inlineStr"/>
-      <c r="AY19" s="18" t="inlineStr"/>
-      <c r="AZ19" s="18" t="inlineStr"/>
-      <c r="BA19" s="18" t="inlineStr"/>
-      <c r="BB19" s="18" t="inlineStr"/>
-      <c r="BC19" s="18" t="inlineStr"/>
-      <c r="BD19" s="18" t="inlineStr"/>
-      <c r="BE19" s="18" t="inlineStr"/>
-      <c r="BF19" s="19" t="inlineStr"/>
-      <c r="BG19" s="19" t="inlineStr"/>
-      <c r="BH19" s="19" t="inlineStr"/>
-      <c r="BI19" s="19" t="inlineStr"/>
-      <c r="BJ19" s="19" t="inlineStr"/>
-      <c r="BK19" s="19" t="inlineStr"/>
-      <c r="BL19" s="19" t="inlineStr"/>
-      <c r="BM19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="BN19" t="n">
-        <v>0.304</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>C007</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Simone</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Coordenador</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>100001</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>PROD100002</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Produto de Teste - Processo 100002</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>SSO</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Detector Portátil</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>MicroClip</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>50</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N20" s="11" t="n">
-        <v>0.6320000000000001</v>
-      </c>
-      <c r="O20" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P20" s="12" t="n">
-        <v>120</v>
-      </c>
-      <c r="Q20" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R20" s="12" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="S20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="T20" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="U20" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V20" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="W20" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X20" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Y20" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="Z20" s="13" t="n">
-        <v>0.08000000000000002</v>
-      </c>
-      <c r="AA20" s="14" t="inlineStr"/>
-      <c r="AB20" s="14" t="inlineStr"/>
-      <c r="AC20" s="14" t="inlineStr"/>
-      <c r="AD20" s="14" t="inlineStr"/>
-      <c r="AE20" s="14" t="inlineStr"/>
-      <c r="AF20" s="14" t="inlineStr"/>
-      <c r="AG20" s="15" t="inlineStr"/>
-      <c r="AH20" s="15" t="inlineStr"/>
-      <c r="AI20" s="15" t="inlineStr"/>
-      <c r="AJ20" s="15" t="inlineStr"/>
-      <c r="AK20" s="15" t="inlineStr"/>
-      <c r="AL20" s="15" t="inlineStr"/>
-      <c r="AM20" s="16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AN20" s="16" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="AO20" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP20" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AQ20" s="16" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AR20" s="16" t="n">
-        <v>0.152</v>
-      </c>
-      <c r="AS20" s="17" t="inlineStr"/>
-      <c r="AT20" s="17" t="inlineStr"/>
-      <c r="AU20" s="17" t="inlineStr"/>
-      <c r="AV20" s="17" t="inlineStr"/>
-      <c r="AW20" s="17" t="inlineStr"/>
-      <c r="AX20" s="17" t="inlineStr"/>
-      <c r="AY20" s="18" t="inlineStr"/>
-      <c r="AZ20" s="18" t="inlineStr"/>
-      <c r="BA20" s="18" t="inlineStr"/>
-      <c r="BB20" s="18" t="inlineStr"/>
-      <c r="BC20" s="18" t="inlineStr"/>
-      <c r="BD20" s="18" t="inlineStr"/>
-      <c r="BE20" s="18" t="inlineStr"/>
-      <c r="BF20" s="19" t="inlineStr"/>
-      <c r="BG20" s="19" t="inlineStr"/>
-      <c r="BH20" s="19" t="inlineStr"/>
-      <c r="BI20" s="19" t="inlineStr"/>
-      <c r="BJ20" s="19" t="inlineStr"/>
-      <c r="BK20" s="19" t="inlineStr"/>
-      <c r="BL20" s="19" t="inlineStr"/>
-      <c r="BM20" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="BN20" t="n">
-        <v>0.3160000000000001</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>C008</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Andrey Andrade</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Consultor Interno</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>100001</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>PROD100002</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Produto de Teste - Processo 100002</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>SSO</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Detector Portátil</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>MicroClip</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>50</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N21" s="11" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="O21" s="12" t="inlineStr"/>
-      <c r="P21" s="12" t="inlineStr"/>
-      <c r="Q21" s="12" t="inlineStr"/>
-      <c r="R21" s="12" t="inlineStr"/>
-      <c r="S21" s="12" t="inlineStr"/>
-      <c r="T21" s="12" t="inlineStr"/>
-      <c r="U21" s="13" t="inlineStr"/>
-      <c r="V21" s="13" t="inlineStr"/>
-      <c r="W21" s="13" t="inlineStr"/>
-      <c r="X21" s="13" t="inlineStr"/>
-      <c r="Y21" s="13" t="inlineStr"/>
-      <c r="Z21" s="13" t="inlineStr"/>
-      <c r="AA21" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AB21" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="AC21" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="AD21" s="14" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="AE21" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF21" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AG21" s="15" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AH21" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="AI21" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ21" s="15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AK21" s="15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AL21" s="15" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AM21" s="16" t="inlineStr"/>
-      <c r="AN21" s="16" t="inlineStr"/>
-      <c r="AO21" s="16" t="inlineStr"/>
-      <c r="AP21" s="16" t="inlineStr"/>
-      <c r="AQ21" s="16" t="inlineStr"/>
-      <c r="AR21" s="16" t="inlineStr"/>
-      <c r="AS21" s="17" t="inlineStr"/>
-      <c r="AT21" s="17" t="inlineStr"/>
-      <c r="AU21" s="17" t="inlineStr"/>
-      <c r="AV21" s="17" t="inlineStr"/>
-      <c r="AW21" s="17" t="inlineStr"/>
-      <c r="AX21" s="17" t="inlineStr"/>
-      <c r="AY21" s="18" t="inlineStr"/>
-      <c r="AZ21" s="18" t="inlineStr"/>
-      <c r="BA21" s="18" t="inlineStr"/>
-      <c r="BB21" s="18" t="inlineStr"/>
-      <c r="BC21" s="18" t="inlineStr"/>
-      <c r="BD21" s="18" t="inlineStr"/>
-      <c r="BE21" s="18" t="inlineStr"/>
-      <c r="BF21" s="19" t="inlineStr"/>
-      <c r="BG21" s="19" t="inlineStr"/>
-      <c r="BH21" s="19" t="inlineStr"/>
-      <c r="BI21" s="19" t="inlineStr"/>
-      <c r="BJ21" s="19" t="inlineStr"/>
-      <c r="BK21" s="19" t="inlineStr"/>
-      <c r="BL21" s="19" t="inlineStr"/>
-      <c r="BM21" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="BN21" t="n">
-        <v>0.195</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>C015</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>André Camargo</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Consultor Externo</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>100001</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>PROD100002</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Produto de Teste - Processo 100002</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>SSO</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Detector Portátil</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>MicroClip</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>50</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N22" s="11" t="n">
-        <v>0.6799999999999999</v>
-      </c>
-      <c r="O22" s="12" t="inlineStr"/>
-      <c r="P22" s="12" t="inlineStr"/>
-      <c r="Q22" s="12" t="inlineStr"/>
-      <c r="R22" s="12" t="inlineStr"/>
-      <c r="S22" s="12" t="inlineStr"/>
-      <c r="T22" s="12" t="inlineStr"/>
-      <c r="U22" s="13" t="inlineStr"/>
-      <c r="V22" s="13" t="inlineStr"/>
-      <c r="W22" s="13" t="inlineStr"/>
-      <c r="X22" s="13" t="inlineStr"/>
-      <c r="Y22" s="13" t="inlineStr"/>
-      <c r="Z22" s="13" t="inlineStr"/>
-      <c r="AA22" s="14" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AB22" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="AC22" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="AD22" s="14" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="AE22" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF22" s="14" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AG22" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AH22" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="AI22" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ22" s="15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AK22" s="15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AL22" s="15" t="n">
-        <v>0.08000000000000002</v>
-      </c>
-      <c r="AM22" s="16" t="inlineStr"/>
-      <c r="AN22" s="16" t="inlineStr"/>
-      <c r="AO22" s="16" t="inlineStr"/>
-      <c r="AP22" s="16" t="inlineStr"/>
-      <c r="AQ22" s="16" t="inlineStr"/>
-      <c r="AR22" s="16" t="inlineStr"/>
-      <c r="AS22" s="17" t="inlineStr"/>
-      <c r="AT22" s="17" t="inlineStr"/>
-      <c r="AU22" s="17" t="inlineStr"/>
-      <c r="AV22" s="17" t="inlineStr"/>
-      <c r="AW22" s="17" t="inlineStr"/>
-      <c r="AX22" s="17" t="inlineStr"/>
-      <c r="AY22" s="18" t="inlineStr"/>
-      <c r="AZ22" s="18" t="inlineStr"/>
-      <c r="BA22" s="18" t="inlineStr"/>
-      <c r="BB22" s="18" t="inlineStr"/>
-      <c r="BC22" s="18" t="inlineStr"/>
-      <c r="BD22" s="18" t="inlineStr"/>
-      <c r="BE22" s="18" t="inlineStr"/>
-      <c r="BF22" s="19" t="inlineStr"/>
-      <c r="BG22" s="19" t="inlineStr"/>
-      <c r="BH22" s="19" t="inlineStr"/>
-      <c r="BI22" s="19" t="inlineStr"/>
-      <c r="BJ22" s="19" t="inlineStr"/>
-      <c r="BK22" s="19" t="inlineStr"/>
-      <c r="BL22" s="19" t="inlineStr"/>
-      <c r="BM22" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="BN22" t="n">
-        <v>0.255</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4158,7 +3412,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.5615</v>
+        <v>0.3475</v>
       </c>
     </row>
     <row r="3">
@@ -4178,7 +3432,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.027</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="4">
@@ -4258,7 +3512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.12</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="8">
@@ -4278,7 +3532,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.468</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="9">
@@ -4418,7 +3672,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.312</v>
+        <v>0.9625000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -4532,7 +3786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4582,7 +3836,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': '100002'}</t>
+          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': 100002}</t>
         </is>
       </c>
     </row>
@@ -4599,7 +3853,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': '100002'}</t>
+          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': 100002}</t>
         </is>
       </c>
     </row>
@@ -4645,12 +3899,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rentabilidade não encontrada para chave ('SSO', 'Detector Fixo', 'XCD', 'Produto') (item: PROD100002)</t>
+          <t>Rentabilidade não encontrada para chave ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto') (item: PROD400001)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': 100002}</t>
+          <t>{'chave_busca': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'chave_original': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'item': 'PROD400001', 'processo': 400001}</t>
         </is>
       </c>
     </row>
@@ -4662,12 +3916,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rentabilidade não encontrada para chave ('SSO', 'Detector Fixo', 'XCD', 'Produto') (item: PROD100002)</t>
+          <t>Rentabilidade não encontrada para chave ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto') (item: PROD400001)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{'chave_busca': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'chave_original': ('SSO', 'Detector Fixo', 'XCD', 'Produto'), 'item': 'PROD100002', 'processo': 100002}</t>
+          <t>{'chave_busca': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'chave_original': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'item': 'PROD400001', 'processo': 400001}</t>
         </is>
       </c>
     </row>
@@ -4713,12 +3967,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Rentabilidade não encontrada para chave ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto') (item: PROD400001)</t>
+          <t>Meta não encontrada para tipo 'faturamento_individual' e chave 'Mateus Machado'.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{'chave_busca': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'chave_original': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'item': 'PROD400001', 'processo': 400001}</t>
+          <t>{'tipo_meta': 'faturamento_individual', 'chave': 'Mateus Machado', 'erro': 'single positional indexer is out-of-bounds'}</t>
         </is>
       </c>
     </row>
@@ -4730,44 +3984,10 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Rentabilidade não encontrada para chave ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto') (item: PROD400001)</t>
+          <t>Meta não encontrada para tipo 'conversao_individual' e chave 'Mateus Machado'.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
-        <is>
-          <t>{'chave_busca': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'chave_original': ('Hidrologia', 'Medidor de Vazão Fixo', 'ADP', 'Produto'), 'item': 'PROD400001', 'processo': 400001}</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>AVISO</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Meta não encontrada para tipo 'faturamento_individual' e chave 'Mateus Machado'.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>{'tipo_meta': 'faturamento_individual', 'chave': 'Mateus Machado', 'erro': 'single positional indexer is out-of-bounds'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>AVISO</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Meta não encontrada para tipo 'conversao_individual' e chave 'Mateus Machado'.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
         <is>
           <t>{'tipo_meta': 'conversao_individual', 'chave': 'Mateus Machado', 'erro': 'single positional indexer is out-of-bounds'}</t>
         </is>
@@ -5146,7 +4366,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>André Caramello</t>
+          <t>Alessandro Cappi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5156,12 +4376,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PROD400001</t>
+          <t>PROD100002</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Hidrologia</t>
+          <t>SSO</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -5169,12 +4389,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ISCO</t>
+          <t>ION</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -5223,7 +4443,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Alessandro Cappi</t>
+          <t>André Caramello</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5233,12 +4453,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PROD100002</t>
+          <t>PROD400001</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SSO</t>
+          <t>Hidrologia</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -5246,12 +4466,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ION</t>
+          <t>ISCO</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -5367,7 +4587,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-12-03T16:46:23.690573</t>
+          <t>2025-12-04T15:08:34.340821</t>
         </is>
       </c>
     </row>

</xml_diff>